<commit_message>
persisting puzzle config in sqlite, domain events refactoring
</commit_message>
<xml_diff>
--- a/docs/perfect_pitch_app_plan.xlsx
+++ b/docs/perfect_pitch_app_plan.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Sheet4" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Sheet5" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Sheet6" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="219">
   <si>
     <t xml:space="preserve">Thing to learn</t>
   </si>
@@ -299,6 +301,15 @@
     <t xml:space="preserve">note or not? the mode where you configure several notes, and target note. the puzzle is to guess whether is currently sounding note is the target note or not.</t>
   </si>
   <si>
+    <t xml:space="preserve">percentage of successful octave guesses, of successful note in octave guesses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">different sounds of notes. e.g.: piano/saxophone/flute/vocal note from song sounds on piano keyboard key pressing. randomly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">use keyboard play/stop key (kinda custom, at least it exists not on all keyboards) to replay hint. jsut for fun</t>
+  </si>
+  <si>
     <t xml:space="preserve">JAVA LEARNING</t>
   </si>
   <si>
@@ -345,7 +356,7 @@
     <t xml:space="preserve">vavr lib (functional lib)</t>
   </si>
   <si>
-    <t xml:space="preserve">using &lt;?&gt; instad of &lt;T&gt;</t>
+    <t xml:space="preserve">using &lt;?&gt; instead of &lt;T&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">syntactic sugar</t>
@@ -375,6 +386,27 @@
     <t xml:space="preserve">distributed transaction</t>
   </si>
   <si>
+    <t xml:space="preserve">JavaBean is who</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dao is what</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JDBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">difference between Component and Service in spring boot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sort out Spring questions, di, tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oauth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">logging in spring</t>
+  </si>
+  <si>
     <t xml:space="preserve">vlad khononov</t>
   </si>
   <si>
@@ -445,15 +477,234 @@
   </si>
   <si>
     <t xml:space="preserve">turned out yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sessionStarted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8e645458-7de7-4053-b48f-e6a30ffa2927</t>
+  </si>
+  <si>
+    <t xml:space="preserve">org.swetlokognatsk.earking_out.core.domain.events.session.SessionStartedEvent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:45:07.902190785</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:45:07.693181458","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">newPuzzleCreated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">org.swetlokognatsk.earking_out.core.domain.events.session.NewPuzzleCreatedEvent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:45:29.027265516</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:45:07.70255815","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":28}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">repeatHint x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">org.swetlokognatsk.earking_out.core.domain.events.session.UserTriedToGuessPuzzleEvent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:01.893920029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:01.889853653","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":1,"guess":{"keyNumber":{"octaveScopedKeyNumber":1,"value":28}},"attempt":1,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (success)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:01.901797532</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:01.890909433","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":32}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:20.349290525</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:20.345831664","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":2,"guess":{"keyNumber":{"octaveScopedKeyNumber":5,"value":32}},"attempt":1,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:20.355473473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:20.346635119","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":31}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:32.311121902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:32.308403107","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":3,"guess":{"keyNumber":{"octaveScopedKeyNumber":3,"value":30}},"attempt":1,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guess (fail)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:53.714791394</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:53.70100276","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":3,"guess":{"keyNumber":{"octaveScopedKeyNumber":4,"value":31}},"attempt":2,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">repeatHint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:47:53.731509038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:47:53.704433423","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":30}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:11.514565765</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:11.505210551","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":4,"guess":{"keyNumber":{"octaveScopedKeyNumber":2,"value":29}},"attempt":1,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:19.861344072</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:19.857832424","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":4,"guess":{"keyNumber":{"octaveScopedKeyNumber":1,"value":28}},"attempt":2,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:26.748247178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:26.743873938","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":4,"guess":{"keyNumber":{"octaveScopedKeyNumber":2,"value":29}},"attempt":3,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:28.121138238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:28.111252943","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":4,"guess":{"keyNumber":{"octaveScopedKeyNumber":1,"value":28}},"attempt":4,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:34.805303062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:34.792379886","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":4,"guess":{"keyNumber":{"octaveScopedKeyNumber":3,"value":30}},"attempt":5,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:34.820552545</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:34.79535066","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":29}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:43.690996094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:43.688132163","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":5,"guess":{"keyNumber":{"octaveScopedKeyNumber":1,"value":28}},"attempt":1,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:48.422968104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:48.410179585","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":5,"guess":{"keyNumber":{"octaveScopedKeyNumber":2,"value":29}},"attempt":2,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:48.44101343</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:48.41336786","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":31}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:52.858312357</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:52.84464636","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":6,"guess":{"keyNumber":{"octaveScopedKeyNumber":4,"value":31}},"attempt":1,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:52.887326773</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:52.848109785","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":30}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:57.351663043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:57.342907908","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":7,"guess":{"keyNumber":{"octaveScopedKeyNumber":3,"value":30}},"attempt":1,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:48:57.358614452</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:48:57.343704556","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":28}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:08.262641328</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:08.259241449","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":8,"guess":{"keyNumber":{"octaveScopedKeyNumber":2,"value":29}},"attempt":1,"success":false}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:14.010318985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:14.004023478","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":8,"guess":{"keyNumber":{"octaveScopedKeyNumber":1,"value":28}},"attempt":2,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:14.018336321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:14.006584773","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":32}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:20.442782634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:20.430516121","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":9,"guess":{"keyNumber":{"octaveScopedKeyNumber":5,"value":32}},"attempt":1,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:20.467479531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:20.433288272","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzle":{"exercise":{"name":"PERFECT_PITCH","type":"AUDIO"},"solution":{"keyNumber":{"octaveScopedKeyNumber":0,"value":32}}}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:32.130195902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:32.122228279","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"},"puzzleNumber":10,"guess":{"keyNumber":{"octaveScopedKeyNumber":5,"value":32}},"attempt":1,"success":true}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">org.swetlokognatsk.earking_out.core.domain.events.session.SessionFinishedEvent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-06T14:49:32.146492293</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"timestamp":"2026-08-06T14:49:32.122289839","sessionId":{"id":"8e645458-7de7-4053-b48f-e6a30ffa2927"}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 of 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sessionFinished</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
+    <numFmt numFmtId="166" formatCode="hh:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="167" formatCode="@"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -502,7 +753,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -571,6 +822,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
+        <bgColor rgb="FF999999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF999999"/>
+        <bgColor rgb="FFAFABAB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.25"/>
         <bgColor rgb="FFAFABAB"/>
       </patternFill>
@@ -590,7 +853,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF5983B0"/>
-        <bgColor rgb="FF3366FF"/>
+        <bgColor rgb="FF808080"/>
       </patternFill>
     </fill>
     <fill>
@@ -653,7 +916,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -722,10 +985,22 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -738,7 +1013,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -754,7 +1029,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -762,23 +1037,47 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -808,8 +1107,8 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF77BC65"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FFAFABAB"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
@@ -834,13 +1133,13 @@
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF77BC65"/>
       <rgbColor rgb="FFBBE33D"/>
       <rgbColor rgb="FFFFC000"/>
       <rgbColor rgb="FFFF8000"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF5983B0"/>
-      <rgbColor rgb="FFAFABAB"/>
+      <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF00B050"/>
       <rgbColor rgb="FF003300"/>
@@ -1136,7 +1435,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D109"/>
+  <dimension ref="A1:D116"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="81.39"/>
@@ -1300,7 +1599,7 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="9" t="s">
         <v>49</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1308,7 +1607,7 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="9" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1318,17 +1617,17 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="17" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="18" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B25" s="13" t="s">
@@ -1336,7 +1635,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="20" t="s">
         <v>55</v>
       </c>
       <c r="C26" s="4"/>
@@ -1347,11 +1646,11 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
     </row>
     <row r="30" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
@@ -1364,7 +1663,7 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="90.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="18" t="s">
         <v>60</v>
       </c>
       <c r="D32" s="13" t="s">
@@ -1372,7 +1671,7 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="19" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1382,11 +1681,11 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="19" t="s">
+      <c r="A38" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
+      <c r="B38" s="22"/>
+      <c r="C38" s="22"/>
     </row>
     <row r="40" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
@@ -1397,7 +1696,7 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="9" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1407,11 +1706,11 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="19" t="s">
+      <c r="A46" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
     </row>
     <row r="47" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
@@ -1449,11 +1748,11 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="B59" s="19"/>
-      <c r="C59" s="19"/>
+      <c r="B59" s="22"/>
+      <c r="C59" s="22"/>
     </row>
     <row r="60" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
@@ -1466,7 +1765,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="20" t="s">
+      <c r="A62" s="23" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1506,140 +1805,146 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="21" t="s">
+      <c r="A70" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="B70" s="21"/>
-      <c r="C70" s="21"/>
-    </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="21"/>
-      <c r="B71" s="21"/>
-      <c r="C71" s="21"/>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="21"/>
-      <c r="B72" s="21"/>
-      <c r="C72" s="21"/>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="21"/>
-      <c r="B73" s="21"/>
-      <c r="C73" s="21"/>
+      <c r="B70" s="24"/>
+      <c r="C70" s="24"/>
+    </row>
+    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B71" s="24"/>
+      <c r="C71" s="24"/>
+    </row>
+    <row r="72" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B72" s="24"/>
+      <c r="C72" s="24"/>
+    </row>
+    <row r="73" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B73" s="24"/>
+      <c r="C73" s="24"/>
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="21"/>
-      <c r="B74" s="21"/>
-      <c r="C74" s="21"/>
+      <c r="A74" s="24"/>
+      <c r="B74" s="24"/>
+      <c r="C74" s="24"/>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="21"/>
-      <c r="B75" s="21"/>
-      <c r="C75" s="21"/>
+      <c r="A75" s="24"/>
+      <c r="B75" s="24"/>
+      <c r="C75" s="24"/>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="21"/>
-      <c r="B76" s="21"/>
-      <c r="C76" s="21"/>
+      <c r="A76" s="24"/>
+      <c r="B76" s="24"/>
+      <c r="C76" s="24"/>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="21"/>
-      <c r="B77" s="21"/>
-      <c r="C77" s="21"/>
+      <c r="A77" s="24"/>
+      <c r="B77" s="24"/>
+      <c r="C77" s="24"/>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="21"/>
-      <c r="B78" s="21"/>
-      <c r="C78" s="21"/>
+      <c r="A78" s="24"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="24"/>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="21"/>
-      <c r="B79" s="21"/>
-      <c r="C79" s="21"/>
+      <c r="A79" s="24"/>
+      <c r="B79" s="24"/>
+      <c r="C79" s="24"/>
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="21"/>
-      <c r="B80" s="21"/>
-      <c r="C80" s="21"/>
+      <c r="A80" s="24"/>
+      <c r="B80" s="24"/>
+      <c r="C80" s="24"/>
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="21"/>
-      <c r="B81" s="21"/>
-      <c r="C81" s="21"/>
+      <c r="A81" s="24"/>
+      <c r="B81" s="24"/>
+      <c r="C81" s="24"/>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="21"/>
-      <c r="B82" s="21"/>
-      <c r="C82" s="21"/>
+      <c r="A82" s="24"/>
+      <c r="B82" s="24"/>
+      <c r="C82" s="24"/>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="21"/>
-      <c r="B83" s="21"/>
-      <c r="C83" s="21"/>
+      <c r="A83" s="24"/>
+      <c r="B83" s="24"/>
+      <c r="C83" s="24"/>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="21"/>
-      <c r="B84" s="21"/>
-      <c r="C84" s="21"/>
+      <c r="A84" s="24"/>
+      <c r="B84" s="24"/>
+      <c r="C84" s="24"/>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="21"/>
-      <c r="B85" s="21"/>
-      <c r="C85" s="21"/>
+      <c r="A85" s="24"/>
+      <c r="B85" s="24"/>
+      <c r="C85" s="24"/>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="21"/>
-      <c r="B86" s="21"/>
-      <c r="C86" s="21"/>
+      <c r="A86" s="24"/>
+      <c r="B86" s="24"/>
+      <c r="C86" s="24"/>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="21"/>
-      <c r="B87" s="21"/>
-      <c r="C87" s="21"/>
+      <c r="A87" s="24"/>
+      <c r="B87" s="24"/>
+      <c r="C87" s="24"/>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="21"/>
-      <c r="B88" s="21"/>
-      <c r="C88" s="21"/>
+      <c r="A88" s="24"/>
+      <c r="B88" s="24"/>
+      <c r="C88" s="24"/>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="21"/>
-      <c r="B89" s="21"/>
-      <c r="C89" s="21"/>
+      <c r="A89" s="24"/>
+      <c r="B89" s="24"/>
+      <c r="C89" s="24"/>
     </row>
     <row r="90" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="B90" s="18"/>
-      <c r="C90" s="18"/>
+      <c r="A90" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="21"/>
+      <c r="C90" s="21"/>
     </row>
     <row r="91" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="22" t="s">
-        <v>95</v>
+      <c r="A95" s="25" t="s">
+        <v>98</v>
       </c>
       <c r="B95" s="12" t="n">
         <v>0.5</v>
@@ -1647,81 +1952,116 @@
     </row>
     <row r="96" customFormat="false" ht="75.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="105.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="9" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="15" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1754,58 +2094,58 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="23" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="23" width="33.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="23" width="28.39"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="23" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="26" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="26" width="33.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="26" width="28.39"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="26" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24"/>
-      <c r="B1" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>115</v>
+      <c r="A1" s="27"/>
+      <c r="B1" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="120.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>118</v>
+      <c r="A2" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>121</v>
+      <c r="A4" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>124</v>
+      <c r="A5" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1839,162 +2179,162 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="28" t="s">
-        <v>134</v>
-      </c>
-      <c r="I2" s="28" t="s">
-        <v>134</v>
+        <v>135</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="I2" s="31" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
+        <v>136</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="E4" s="30"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="I4" s="31" t="s">
-        <v>135</v>
+      <c r="A4" s="32" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="E4" s="33"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="I4" s="34" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="27"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
+        <v>130</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="F5" s="30"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="G6" s="27"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
+        <v>126</v>
+      </c>
+      <c r="B6" s="30"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
+        <v>138</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="26" t="s">
-        <v>136</v>
-      </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="I8" s="26"/>
+        <v>139</v>
+      </c>
+      <c r="B8" s="30"/>
+      <c r="C8" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="I8" s="29"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="25" t="s">
-        <v>131</v>
+        <v>140</v>
+      </c>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="28" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2008,4 +2348,614 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E1" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="1.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="38.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="80.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="112.65"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="37" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E2" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" s="39" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E3" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3" s="39" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="38" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F4" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="G4" s="38" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F5" s="39" t="s">
+        <v>162</v>
+      </c>
+      <c r="G5" s="38" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F6" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="G6" s="38" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="G7" s="38" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>168</v>
+      </c>
+      <c r="G8" s="38" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E9" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F9" s="39" t="s">
+        <v>171</v>
+      </c>
+      <c r="G9" s="38" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F10" s="39" t="s">
+        <v>174</v>
+      </c>
+      <c r="G10" s="38" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F11" s="39" t="s">
+        <v>176</v>
+      </c>
+      <c r="G11" s="38" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="G12" s="38" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F13" s="39" t="s">
+        <v>180</v>
+      </c>
+      <c r="G13" s="38" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F14" s="39" t="s">
+        <v>182</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D15" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F15" s="39" t="s">
+        <v>184</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F16" s="39" t="s">
+        <v>186</v>
+      </c>
+      <c r="G16" s="38" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D17" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E17" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F17" s="39" t="s">
+        <v>188</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F18" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F19" s="39" t="s">
+        <v>192</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F20" s="39" t="s">
+        <v>194</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F21" s="39" t="s">
+        <v>196</v>
+      </c>
+      <c r="G21" s="38" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F22" s="39" t="s">
+        <v>198</v>
+      </c>
+      <c r="G22" s="38" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F23" s="39" t="s">
+        <v>200</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E24" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F24" s="39" t="s">
+        <v>202</v>
+      </c>
+      <c r="G24" s="38" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F25" s="39" t="s">
+        <v>204</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F26" s="39" t="s">
+        <v>206</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E27" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F27" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="G27" s="38" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E28" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="F28" s="39" t="s">
+        <v>210</v>
+      </c>
+      <c r="G28" s="38" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E29" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="F29" s="39" t="s">
+        <v>212</v>
+      </c>
+      <c r="G29" s="38" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="E30" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="F30" s="39" t="s">
+        <v>215</v>
+      </c>
+      <c r="G30" s="38" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B34" s="40" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
git cleaning, some docs
</commit_message>
<xml_diff>
--- a/docs/perfect_pitch_app_plan.xlsx
+++ b/docs/perfect_pitch_app_plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="225">
   <si>
     <t xml:space="preserve">Thing to learn</t>
   </si>
@@ -262,9 +262,6 @@
     <t xml:space="preserve">implement psql adapter</t>
   </si>
   <si>
-    <t xml:space="preserve">what to do with UserId? how to access it and attach to event if service layer and domain core is shared for both desktop and web version (there's no UserId in desktop version)</t>
-  </si>
-  <si>
     <t xml:space="preserve">INTERESTING IDEAS</t>
   </si>
   <si>
@@ -307,7 +304,13 @@
     <t xml:space="preserve">different sounds of notes. e.g.: piano/saxophone/flute/vocal note from song sounds on piano keyboard key pressing. randomly.</t>
   </si>
   <si>
-    <t xml:space="preserve">use keyboard play/stop key (kinda custom, at least it exists not on all keyboards) to replay hint. jsut for fun</t>
+    <t xml:space="preserve">use computer keyboard play/stop key (kinda custom, at least it exists not on all keyboards) to replay hint. jsut for fun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer (notes per second?)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marathon - continuous gussing until user reaches specified percentage (e.g. 90%)</t>
   </si>
   <si>
     <t xml:space="preserve">JAVA LEARNING</t>
@@ -422,7 +425,7 @@
     <t xml:space="preserve">= entity. has public read-only state. the state can only be changed via methods, by aggregate itself. These methods enforce validation and consistency. works on data in-memory. when everything is fine, service saves aggregate using repository</t>
   </si>
   <si>
-    <t xml:space="preserve">works on in-storage data</t>
+    <t xml:space="preserve">works on in-memory data</t>
   </si>
   <si>
     <t xml:space="preserve">aggregate root</t>
@@ -477,6 +480,21 @@
   </si>
   <si>
     <t xml:space="preserve">turned out yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMPORTANT THINGS TO DO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">java ORMs (Hibernate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">event sourcing logging via tasks/threads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">web UI (Spring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CQRS via statistics</t>
   </si>
   <si>
     <t xml:space="preserve">14 45</t>
@@ -753,12 +771,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF00B050"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -782,12 +806,6 @@
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.25"/>
         <bgColor rgb="FFBFBFBF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00A933"/>
-        <bgColor rgb="FF00B050"/>
       </patternFill>
     </fill>
     <fill>
@@ -840,14 +858,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF4000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF993300"/>
+        <fgColor rgb="FFFF4000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF6D"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
     <fill>
@@ -865,13 +895,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF8000"/>
-        <bgColor rgb="FFFF6600"/>
+        <bgColor rgb="FFFF8080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFBBE33D"/>
         <bgColor rgb="FFA9D18E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF729FCF"/>
+        <bgColor rgb="FF5983B0"/>
       </patternFill>
     </fill>
   </fills>
@@ -916,7 +952,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -929,6 +965,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -937,26 +977,26 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1005,11 +1045,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1021,6 +1065,18 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1029,11 +1085,23 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1041,28 +1109,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="21" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="23" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1108,7 +1160,7 @@
       <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FFAFABAB"/>
+      <rgbColor rgb="FF729FCF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
@@ -1127,17 +1179,17 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFC5E0B4"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFFF6D"/>
       <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFAFABAB"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF77BC65"/>
       <rgbColor rgb="FFBBE33D"/>
       <rgbColor rgb="FFFFC000"/>
       <rgbColor rgb="FFFF8000"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFFF4000"/>
       <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
@@ -1346,10 +1398,10 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1362,26 +1414,26 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1394,18 +1446,18 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1438,630 +1490,632 @@
   <dimension ref="A1:D116"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="81.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="29.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="23.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="92.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="101.28"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="3" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="81.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="29.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="23.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="92.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="101.28"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="4" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="D3" s="3" t="s">
+      <c r="B3" s="8"/>
+      <c r="D3" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="60.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="4"/>
+      <c r="D16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="12" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="16" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="17" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="18" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="19" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
     </row>
     <row r="30" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="7" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="90.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="14" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="20" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="23" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="14" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="s">
+      <c r="A41" s="10" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="10" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="22" t="s">
+      <c r="A46" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="24"/>
     </row>
     <row r="47" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="23" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1"/>
+    </row>
+    <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="24" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="22" t="s">
+      <c r="B59" s="24"/>
+      <c r="C59" s="24"/>
+    </row>
+    <row r="60" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B59" s="22"/>
-      <c r="C59" s="22"/>
-    </row>
-    <row r="60" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
+    </row>
+    <row r="61" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="23" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+    <row r="62" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="25" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="23" t="s">
+    <row r="63" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
+    <row r="64" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3" t="s">
+    <row r="65" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
+    <row r="66" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="3" t="s">
+    <row r="67" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
+    <row r="68" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="23" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
+    <row r="69" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3" t="s">
+    <row r="70" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="26" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="70" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="24" t="s">
+      <c r="B70" s="26"/>
+      <c r="C70" s="26"/>
+    </row>
+    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B70" s="24"/>
-      <c r="C70" s="24"/>
-    </row>
-    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="24" t="s">
+      <c r="B71" s="26"/>
+      <c r="C71" s="26"/>
+    </row>
+    <row r="72" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B71" s="24"/>
-      <c r="C71" s="24"/>
-    </row>
-    <row r="72" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="24" t="s">
+      <c r="B72" s="26"/>
+      <c r="C72" s="26"/>
+    </row>
+    <row r="73" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B72" s="24"/>
-      <c r="C72" s="24"/>
-    </row>
-    <row r="73" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="3" t="s">
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+    </row>
+    <row r="74" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="24"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="24"/>
-      <c r="B75" s="24"/>
-      <c r="C75" s="24"/>
+      <c r="B74" s="26"/>
+      <c r="C74" s="26"/>
+    </row>
+    <row r="75" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="B75" s="26"/>
+      <c r="C75" s="26"/>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="24"/>
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
+      <c r="A76" s="26"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="26"/>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="24"/>
-      <c r="B77" s="24"/>
-      <c r="C77" s="24"/>
+      <c r="A77" s="26"/>
+      <c r="B77" s="26"/>
+      <c r="C77" s="26"/>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="24"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="24"/>
+      <c r="A78" s="26"/>
+      <c r="B78" s="26"/>
+      <c r="C78" s="26"/>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="24"/>
-      <c r="B79" s="24"/>
-      <c r="C79" s="24"/>
+      <c r="A79" s="26"/>
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="24"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24"/>
+      <c r="A80" s="26"/>
+      <c r="B80" s="26"/>
+      <c r="C80" s="26"/>
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="24"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="24"/>
+      <c r="A81" s="26"/>
+      <c r="B81" s="26"/>
+      <c r="C81" s="26"/>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="24"/>
-      <c r="B82" s="24"/>
-      <c r="C82" s="24"/>
+      <c r="A82" s="26"/>
+      <c r="B82" s="26"/>
+      <c r="C82" s="26"/>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="24"/>
-      <c r="B83" s="24"/>
-      <c r="C83" s="24"/>
+      <c r="A83" s="26"/>
+      <c r="B83" s="26"/>
+      <c r="C83" s="26"/>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="24"/>
-      <c r="B84" s="24"/>
-      <c r="C84" s="24"/>
+      <c r="A84" s="26"/>
+      <c r="B84" s="26"/>
+      <c r="C84" s="26"/>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="24"/>
-      <c r="B85" s="24"/>
-      <c r="C85" s="24"/>
+      <c r="A85" s="26"/>
+      <c r="B85" s="26"/>
+      <c r="C85" s="26"/>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="24"/>
-      <c r="B86" s="24"/>
-      <c r="C86" s="24"/>
+      <c r="A86" s="26"/>
+      <c r="B86" s="26"/>
+      <c r="C86" s="26"/>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="24"/>
-      <c r="B87" s="24"/>
-      <c r="C87" s="24"/>
+      <c r="A87" s="26"/>
+      <c r="B87" s="26"/>
+      <c r="C87" s="26"/>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="24"/>
-      <c r="B88" s="24"/>
-      <c r="C88" s="24"/>
+      <c r="A88" s="26"/>
+      <c r="B88" s="26"/>
+      <c r="C88" s="26"/>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="24"/>
-      <c r="B89" s="24"/>
-      <c r="C89" s="24"/>
+      <c r="A89" s="26"/>
+      <c r="B89" s="26"/>
+      <c r="C89" s="26"/>
     </row>
     <row r="90" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="B90" s="21"/>
-      <c r="C90" s="21"/>
+      <c r="A90" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B90" s="22"/>
+      <c r="C90" s="22"/>
     </row>
     <row r="91" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B91" s="6" t="s">
+      <c r="A91" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="B91" s="7" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="3" t="s">
-        <v>95</v>
+      <c r="A92" s="4" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="5" t="s">
-        <v>96</v>
+      <c r="A93" s="6" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="5" t="s">
-        <v>97</v>
+      <c r="A94" s="6" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="B95" s="12" t="n">
+      <c r="A95" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B95" s="13" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="75.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B96" s="3" t="s">
+      <c r="A96" s="6" t="s">
         <v>100</v>
       </c>
+      <c r="B96" s="4" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="5" t="s">
-        <v>101</v>
+      <c r="A97" s="6" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="105.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B98" s="3" t="s">
+      <c r="A98" s="6" t="s">
         <v>103</v>
       </c>
+      <c r="B98" s="4" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="5" t="s">
-        <v>104</v>
+      <c r="A99" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="3" t="s">
-        <v>105</v>
+      <c r="A100" s="4" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B101" s="3" t="s">
+      <c r="A101" s="6" t="s">
         <v>107</v>
       </c>
+      <c r="B101" s="4" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="5" t="s">
-        <v>108</v>
+      <c r="A102" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="5" t="s">
-        <v>109</v>
+      <c r="A103" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="5" t="s">
-        <v>110</v>
+      <c r="A104" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="9" t="s">
-        <v>111</v>
+      <c r="A105" s="10" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="3" t="s">
-        <v>112</v>
+      <c r="A106" s="23" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="15" t="s">
-        <v>113</v>
+      <c r="A107" s="23" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="3" t="s">
-        <v>114</v>
+      <c r="A108" s="23" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="3" t="s">
-        <v>115</v>
+      <c r="A109" s="23" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="15" t="s">
-        <v>116</v>
+      <c r="A110" s="10" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="3" t="s">
-        <v>117</v>
+      <c r="A111" s="4" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="11" t="s">
-        <v>118</v>
+      <c r="A112" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="3" t="s">
-        <v>119</v>
+      <c r="A113" s="28" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="9" t="s">
-        <v>120</v>
+      <c r="A114" s="10" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="1" t="s">
-        <v>121</v>
+      <c r="A115" s="29" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="3" t="s">
-        <v>122</v>
+      <c r="A116" s="30" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2091,62 +2145,137 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="26" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="26" width="33.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="26" width="28.39"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="26" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="31.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="36.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="23.2"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="31" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="27"/>
-      <c r="B1" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="C1" s="27" t="s">
+      <c r="A1" s="32"/>
+      <c r="B1" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="C1" s="32" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="120.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
+      <c r="D1" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="B2" s="26" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="B2" s="31" t="s">
         <v>128</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="26" t="s">
+      <c r="A4" s="31" t="s">
         <v>131</v>
       </c>
+      <c r="B4" s="31" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="60.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="B5" s="26" t="s">
+      <c r="A5" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="B5" s="31" t="s">
         <v>134</v>
       </c>
+      <c r="C5" s="31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1"/>
+    </row>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4"/>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4"/>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4"/>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="16"/>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4"/>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4"/>
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4"/>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1"/>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2179,162 +2308,162 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="C2" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="31" t="s">
+      <c r="D2" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="I2" s="31" t="s">
-        <v>144</v>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
+        <v>137</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="E4" s="33"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="I4" s="34" t="s">
-        <v>145</v>
+      <c r="A4" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" s="36"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="I4" s="37" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
+        <v>131</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="F5" s="29"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
+        <v>127</v>
+      </c>
+      <c r="B6" s="29"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" s="29"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B7" s="30"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
+        <v>139</v>
+      </c>
+      <c r="B7" s="29"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="I8" s="29"/>
+        <v>140</v>
+      </c>
+      <c r="B8" s="29"/>
+      <c r="C8" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="28" t="s">
         <v>141</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="33" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2355,45 +2484,97 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:A17"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46.92"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="3" style="1" width="10.16"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B1" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="n">
+    <row r="1" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="31" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="29" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="35" t="n">
-        <v>5</v>
-      </c>
-      <c r="F1" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="H1" s="1" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36" t="n">
-        <v>5</v>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="29" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="40" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="40" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="40" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2424,529 +2605,529 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="37" t="s">
-        <v>147</v>
+      <c r="A1" s="41" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D2" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E2" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="F2" s="39" t="s">
-        <v>151</v>
-      </c>
-      <c r="G2" s="38" t="s">
-        <v>152</v>
+        <v>154</v>
+      </c>
+      <c r="D2" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="43" t="s">
+        <v>157</v>
+      </c>
+      <c r="G2" s="42" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E3" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F3" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="42" t="s">
         <v>155</v>
       </c>
-      <c r="G3" s="38" t="s">
-        <v>156</v>
+      <c r="E3" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F4" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="G4" s="38" t="s">
-        <v>160</v>
+        <v>163</v>
+      </c>
+      <c r="D4" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F4" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="G4" s="42" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F5" s="39" t="s">
-        <v>162</v>
-      </c>
-      <c r="G5" s="38" t="s">
-        <v>163</v>
+        <v>167</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F5" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F6" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="42" t="s">
         <v>164</v>
       </c>
-      <c r="G6" s="38" t="s">
-        <v>165</v>
+      <c r="F6" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="G6" s="42" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E7" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F7" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="G7" s="38" t="s">
         <v>167</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F7" s="43" t="s">
+        <v>172</v>
+      </c>
+      <c r="G7" s="42" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D8" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F8" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="G8" s="38" t="s">
-        <v>169</v>
+        <v>159</v>
+      </c>
+      <c r="D8" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E8" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8" s="42" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D9" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F9" s="39" t="s">
-        <v>171</v>
-      </c>
-      <c r="G9" s="38" t="s">
-        <v>172</v>
+        <v>176</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>177</v>
+      </c>
+      <c r="G9" s="42" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D10" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F10" s="39" t="s">
-        <v>174</v>
-      </c>
-      <c r="G10" s="38" t="s">
-        <v>175</v>
+        <v>179</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F10" s="43" t="s">
+        <v>180</v>
+      </c>
+      <c r="G10" s="42" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D11" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F11" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="G11" s="38" t="s">
-        <v>177</v>
+        <v>167</v>
+      </c>
+      <c r="D11" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F11" s="43" t="s">
+        <v>182</v>
+      </c>
+      <c r="G11" s="42" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D12" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E12" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F12" s="39" t="s">
-        <v>178</v>
-      </c>
-      <c r="G12" s="38" t="s">
-        <v>179</v>
+        <v>159</v>
+      </c>
+      <c r="D12" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E12" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F12" s="43" t="s">
+        <v>184</v>
+      </c>
+      <c r="G12" s="42" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D13" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F13" s="39" t="s">
-        <v>180</v>
-      </c>
-      <c r="G13" s="38" t="s">
-        <v>181</v>
+        <v>179</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E13" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F13" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="G13" s="42" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E14" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F14" s="39" t="s">
-        <v>182</v>
-      </c>
-      <c r="G14" s="38" t="s">
-        <v>183</v>
+        <v>176</v>
+      </c>
+      <c r="D14" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E14" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" s="42" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D15" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E15" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F15" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="G15" s="38" t="s">
-        <v>185</v>
+        <v>176</v>
+      </c>
+      <c r="D15" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="G15" s="42" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F16" s="39" t="s">
-        <v>186</v>
-      </c>
-      <c r="G16" s="38" t="s">
-        <v>187</v>
+        <v>179</v>
+      </c>
+      <c r="D16" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F16" s="43" t="s">
+        <v>192</v>
+      </c>
+      <c r="G16" s="42" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D17" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E17" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>189</v>
+        <v>176</v>
+      </c>
+      <c r="D17" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E17" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F17" s="43" t="s">
+        <v>194</v>
+      </c>
+      <c r="G17" s="42" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D18" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E18" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F18" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="G18" s="38" t="s">
-        <v>191</v>
+        <v>176</v>
+      </c>
+      <c r="D18" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E18" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>196</v>
+      </c>
+      <c r="G18" s="42" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D19" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>192</v>
-      </c>
-      <c r="G19" s="38" t="s">
-        <v>193</v>
+        <v>167</v>
+      </c>
+      <c r="D19" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="G19" s="42" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D20" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E20" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F20" s="39" t="s">
-        <v>194</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>195</v>
+        <v>159</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E20" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>200</v>
+      </c>
+      <c r="G20" s="42" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D21" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E21" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F21" s="39" t="s">
-        <v>196</v>
-      </c>
-      <c r="G21" s="38" t="s">
-        <v>197</v>
+        <v>176</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F21" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="G21" s="42" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D22" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E22" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F22" s="39" t="s">
-        <v>198</v>
-      </c>
-      <c r="G22" s="38" t="s">
-        <v>199</v>
+        <v>167</v>
+      </c>
+      <c r="D22" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E22" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>204</v>
+      </c>
+      <c r="G22" s="42" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>200</v>
-      </c>
-      <c r="G23" s="38" t="s">
-        <v>201</v>
+        <v>159</v>
+      </c>
+      <c r="D23" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E23" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>206</v>
+      </c>
+      <c r="G23" s="42" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D24" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E24" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F24" s="39" t="s">
-        <v>202</v>
-      </c>
-      <c r="G24" s="38" t="s">
-        <v>203</v>
+        <v>167</v>
+      </c>
+      <c r="D24" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E24" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F24" s="43" t="s">
+        <v>208</v>
+      </c>
+      <c r="G24" s="42" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E25" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F25" s="39" t="s">
-        <v>204</v>
-      </c>
-      <c r="G25" s="38" t="s">
-        <v>205</v>
+        <v>159</v>
+      </c>
+      <c r="D25" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F25" s="43" t="s">
+        <v>210</v>
+      </c>
+      <c r="G25" s="42" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D26" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E26" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F26" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="G26" s="38" t="s">
-        <v>207</v>
+        <v>167</v>
+      </c>
+      <c r="D26" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E26" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F26" s="43" t="s">
+        <v>212</v>
+      </c>
+      <c r="G26" s="42" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>208</v>
-      </c>
-      <c r="G27" s="38" t="s">
-        <v>209</v>
+        <v>159</v>
+      </c>
+      <c r="D27" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E27" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>214</v>
+      </c>
+      <c r="G27" s="42" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D28" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E28" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="39" t="s">
-        <v>210</v>
-      </c>
-      <c r="G28" s="38" t="s">
-        <v>211</v>
+        <v>179</v>
+      </c>
+      <c r="D28" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E28" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F28" s="43" t="s">
+        <v>216</v>
+      </c>
+      <c r="G28" s="42" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E29" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>212</v>
-      </c>
-      <c r="G29" s="38" t="s">
-        <v>213</v>
+        <v>176</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E29" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" s="43" t="s">
+        <v>218</v>
+      </c>
+      <c r="G29" s="42" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D30" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E30" s="38" t="s">
-        <v>214</v>
-      </c>
-      <c r="F30" s="39" t="s">
-        <v>215</v>
-      </c>
-      <c r="G30" s="38" t="s">
-        <v>216</v>
+        <v>167</v>
+      </c>
+      <c r="D30" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E30" s="42" t="s">
+        <v>220</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="G30" s="42" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="B34" s="40" t="s">
-        <v>217</v>
+        <v>167</v>
+      </c>
+      <c r="B34" s="44" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
puzzle config validating, minor refactoring, cleaning
</commit_message>
<xml_diff>
--- a/docs/perfect_pitch_app_plan.xlsx
+++ b/docs/perfect_pitch_app_plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="225">
   <si>
     <t xml:space="preserve">Thing to learn</t>
   </si>
@@ -262,9 +262,6 @@
     <t xml:space="preserve">implement psql adapter</t>
   </si>
   <si>
-    <t xml:space="preserve">what to do with UserId? how to access it and attach to event if service layer and domain core is shared for both desktop and web version (there's no UserId in desktop version)</t>
-  </si>
-  <si>
     <t xml:space="preserve">INTERESTING IDEAS</t>
   </si>
   <si>
@@ -307,7 +304,13 @@
     <t xml:space="preserve">different sounds of notes. e.g.: piano/saxophone/flute/vocal note from song sounds on piano keyboard key pressing. randomly.</t>
   </si>
   <si>
-    <t xml:space="preserve">use keyboard play/stop key (kinda custom, at least it exists not on all keyboards) to replay hint. jsut for fun</t>
+    <t xml:space="preserve">use computer keyboard play/stop key (kinda custom, at least it exists not on all keyboards) to replay hint. jsut for fun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer (notes per second?)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marathon - continuous gussing until user reaches specified percentage (e.g. 90%)</t>
   </si>
   <si>
     <t xml:space="preserve">JAVA LEARNING</t>
@@ -422,7 +425,7 @@
     <t xml:space="preserve">= entity. has public read-only state. the state can only be changed via methods, by aggregate itself. These methods enforce validation and consistency. works on data in-memory. when everything is fine, service saves aggregate using repository</t>
   </si>
   <si>
-    <t xml:space="preserve">works on in-storage data</t>
+    <t xml:space="preserve">works on in-memory data</t>
   </si>
   <si>
     <t xml:space="preserve">aggregate root</t>
@@ -477,6 +480,21 @@
   </si>
   <si>
     <t xml:space="preserve">turned out yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMPORTANT THINGS TO DO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">java ORMs (Hibernate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">event sourcing logging via tasks/threads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">web UI (Spring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CQRS via statistics</t>
   </si>
   <si>
     <t xml:space="preserve">14 45</t>
@@ -753,12 +771,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF00B050"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -782,12 +806,6 @@
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.25"/>
         <bgColor rgb="FFBFBFBF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00A933"/>
-        <bgColor rgb="FF00B050"/>
       </patternFill>
     </fill>
     <fill>
@@ -840,14 +858,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF4000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF993300"/>
+        <fgColor rgb="FFFF4000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF6D"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
     <fill>
@@ -865,13 +895,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF8000"/>
-        <bgColor rgb="FFFF6600"/>
+        <bgColor rgb="FFFF8080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFBBE33D"/>
         <bgColor rgb="FFA9D18E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF729FCF"/>
+        <bgColor rgb="FF5983B0"/>
       </patternFill>
     </fill>
   </fills>
@@ -916,7 +952,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -929,6 +965,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -937,26 +977,26 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1005,11 +1045,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1021,6 +1065,18 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1029,11 +1085,23 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1041,28 +1109,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="21" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="23" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1108,7 +1160,7 @@
       <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FFAFABAB"/>
+      <rgbColor rgb="FF729FCF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
@@ -1127,17 +1179,17 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFC5E0B4"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFFF6D"/>
       <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFAFABAB"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF77BC65"/>
       <rgbColor rgb="FFBBE33D"/>
       <rgbColor rgb="FFFFC000"/>
       <rgbColor rgb="FFFF8000"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFFF4000"/>
       <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
@@ -1346,10 +1398,10 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1362,26 +1414,26 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1394,18 +1446,18 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1438,630 +1490,632 @@
   <dimension ref="A1:D116"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="81.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="29.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="23.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="92.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="101.28"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="3" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="81.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="29.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="23.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="92.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="101.28"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="4" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="D3" s="3" t="s">
+      <c r="B3" s="8"/>
+      <c r="D3" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="60.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="4"/>
+      <c r="D16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="12" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="16" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="17" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="18" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="19" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="14" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
     </row>
     <row r="30" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="7" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="90.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="14" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="20" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="23" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="14" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="s">
+      <c r="A41" s="10" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="10" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="22" t="s">
+      <c r="A46" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="24"/>
     </row>
     <row r="47" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="23" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1"/>
+    </row>
+    <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="24" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="22" t="s">
+      <c r="B59" s="24"/>
+      <c r="C59" s="24"/>
+    </row>
+    <row r="60" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B59" s="22"/>
-      <c r="C59" s="22"/>
-    </row>
-    <row r="60" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
+    </row>
+    <row r="61" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="23" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+    <row r="62" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="25" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="23" t="s">
+    <row r="63" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
+    <row r="64" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3" t="s">
+    <row r="65" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
+    <row r="66" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="3" t="s">
+    <row r="67" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
+    <row r="68" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="23" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
+    <row r="69" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3" t="s">
+    <row r="70" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="26" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="70" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="24" t="s">
+      <c r="B70" s="26"/>
+      <c r="C70" s="26"/>
+    </row>
+    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B70" s="24"/>
-      <c r="C70" s="24"/>
-    </row>
-    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="24" t="s">
+      <c r="B71" s="26"/>
+      <c r="C71" s="26"/>
+    </row>
+    <row r="72" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B71" s="24"/>
-      <c r="C71" s="24"/>
-    </row>
-    <row r="72" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="24" t="s">
+      <c r="B72" s="26"/>
+      <c r="C72" s="26"/>
+    </row>
+    <row r="73" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B72" s="24"/>
-      <c r="C72" s="24"/>
-    </row>
-    <row r="73" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="3" t="s">
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+    </row>
+    <row r="74" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="24"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="24"/>
-      <c r="B75" s="24"/>
-      <c r="C75" s="24"/>
+      <c r="B74" s="26"/>
+      <c r="C74" s="26"/>
+    </row>
+    <row r="75" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="B75" s="26"/>
+      <c r="C75" s="26"/>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="24"/>
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
+      <c r="A76" s="26"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="26"/>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="24"/>
-      <c r="B77" s="24"/>
-      <c r="C77" s="24"/>
+      <c r="A77" s="26"/>
+      <c r="B77" s="26"/>
+      <c r="C77" s="26"/>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="24"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="24"/>
+      <c r="A78" s="26"/>
+      <c r="B78" s="26"/>
+      <c r="C78" s="26"/>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="24"/>
-      <c r="B79" s="24"/>
-      <c r="C79" s="24"/>
+      <c r="A79" s="26"/>
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="24"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24"/>
+      <c r="A80" s="26"/>
+      <c r="B80" s="26"/>
+      <c r="C80" s="26"/>
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="24"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="24"/>
+      <c r="A81" s="26"/>
+      <c r="B81" s="26"/>
+      <c r="C81" s="26"/>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="24"/>
-      <c r="B82" s="24"/>
-      <c r="C82" s="24"/>
+      <c r="A82" s="26"/>
+      <c r="B82" s="26"/>
+      <c r="C82" s="26"/>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="24"/>
-      <c r="B83" s="24"/>
-      <c r="C83" s="24"/>
+      <c r="A83" s="26"/>
+      <c r="B83" s="26"/>
+      <c r="C83" s="26"/>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="24"/>
-      <c r="B84" s="24"/>
-      <c r="C84" s="24"/>
+      <c r="A84" s="26"/>
+      <c r="B84" s="26"/>
+      <c r="C84" s="26"/>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="24"/>
-      <c r="B85" s="24"/>
-      <c r="C85" s="24"/>
+      <c r="A85" s="26"/>
+      <c r="B85" s="26"/>
+      <c r="C85" s="26"/>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="24"/>
-      <c r="B86" s="24"/>
-      <c r="C86" s="24"/>
+      <c r="A86" s="26"/>
+      <c r="B86" s="26"/>
+      <c r="C86" s="26"/>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="24"/>
-      <c r="B87" s="24"/>
-      <c r="C87" s="24"/>
+      <c r="A87" s="26"/>
+      <c r="B87" s="26"/>
+      <c r="C87" s="26"/>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="24"/>
-      <c r="B88" s="24"/>
-      <c r="C88" s="24"/>
+      <c r="A88" s="26"/>
+      <c r="B88" s="26"/>
+      <c r="C88" s="26"/>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="24"/>
-      <c r="B89" s="24"/>
-      <c r="C89" s="24"/>
+      <c r="A89" s="26"/>
+      <c r="B89" s="26"/>
+      <c r="C89" s="26"/>
     </row>
     <row r="90" customFormat="false" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="B90" s="21"/>
-      <c r="C90" s="21"/>
+      <c r="A90" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B90" s="22"/>
+      <c r="C90" s="22"/>
     </row>
     <row r="91" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B91" s="6" t="s">
+      <c r="A91" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="B91" s="7" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="3" t="s">
-        <v>95</v>
+      <c r="A92" s="4" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="5" t="s">
-        <v>96</v>
+      <c r="A93" s="6" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="5" t="s">
-        <v>97</v>
+      <c r="A94" s="6" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="B95" s="12" t="n">
+      <c r="A95" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B95" s="13" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="75.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B96" s="3" t="s">
+      <c r="A96" s="6" t="s">
         <v>100</v>
       </c>
+      <c r="B96" s="4" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="5" t="s">
-        <v>101</v>
+      <c r="A97" s="6" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="105.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B98" s="3" t="s">
+      <c r="A98" s="6" t="s">
         <v>103</v>
       </c>
+      <c r="B98" s="4" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="5" t="s">
-        <v>104</v>
+      <c r="A99" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="3" t="s">
-        <v>105</v>
+      <c r="A100" s="4" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B101" s="3" t="s">
+      <c r="A101" s="6" t="s">
         <v>107</v>
       </c>
+      <c r="B101" s="4" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="5" t="s">
-        <v>108</v>
+      <c r="A102" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="5" t="s">
-        <v>109</v>
+      <c r="A103" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="5" t="s">
-        <v>110</v>
+      <c r="A104" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="9" t="s">
-        <v>111</v>
+      <c r="A105" s="10" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="3" t="s">
-        <v>112</v>
+      <c r="A106" s="23" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="15" t="s">
-        <v>113</v>
+      <c r="A107" s="23" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="3" t="s">
-        <v>114</v>
+      <c r="A108" s="23" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="3" t="s">
-        <v>115</v>
+      <c r="A109" s="23" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="15" t="s">
-        <v>116</v>
+      <c r="A110" s="10" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="3" t="s">
-        <v>117</v>
+      <c r="A111" s="4" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="11" t="s">
-        <v>118</v>
+      <c r="A112" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="3" t="s">
-        <v>119</v>
+      <c r="A113" s="28" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="9" t="s">
-        <v>120</v>
+      <c r="A114" s="10" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="1" t="s">
-        <v>121</v>
+      <c r="A115" s="29" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="3" t="s">
-        <v>122</v>
+      <c r="A116" s="30" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2091,62 +2145,137 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="26" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="26" width="33.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="26" width="28.39"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="26" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="31.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="36.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="23.2"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="31" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="27"/>
-      <c r="B1" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="C1" s="27" t="s">
+      <c r="A1" s="32"/>
+      <c r="B1" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="C1" s="32" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="120.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
+      <c r="D1" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="B2" s="26" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="B2" s="31" t="s">
         <v>128</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="26" t="s">
+      <c r="A4" s="31" t="s">
         <v>131</v>
       </c>
+      <c r="B4" s="31" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="60.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="B5" s="26" t="s">
+      <c r="A5" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="B5" s="31" t="s">
         <v>134</v>
       </c>
+      <c r="C5" s="31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1"/>
+    </row>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4"/>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4"/>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4"/>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="16"/>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4"/>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4"/>
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4"/>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1"/>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2179,162 +2308,162 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="C2" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="31" t="s">
+      <c r="D2" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="I2" s="31" t="s">
-        <v>144</v>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
+        <v>137</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>137</v>
-      </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="E4" s="33"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="I4" s="34" t="s">
-        <v>145</v>
+      <c r="A4" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" s="36"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="I4" s="37" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
+        <v>131</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="F5" s="29"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
+        <v>127</v>
+      </c>
+      <c r="B6" s="29"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" s="29"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B7" s="30"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
+        <v>139</v>
+      </c>
+      <c r="B7" s="29"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="I8" s="29"/>
+        <v>140</v>
+      </c>
+      <c r="B8" s="29"/>
+      <c r="C8" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="28" t="s">
         <v>141</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="33" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2355,45 +2484,97 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:A17"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46.92"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="3" style="1" width="10.16"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B1" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="n">
+    <row r="1" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="31" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="29" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="35" t="n">
-        <v>5</v>
-      </c>
-      <c r="F1" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="H1" s="1" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36" t="n">
-        <v>5</v>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="29" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="40" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="40" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="40" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2424,529 +2605,529 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="37" t="s">
-        <v>147</v>
+      <c r="A1" s="41" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D2" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E2" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="F2" s="39" t="s">
-        <v>151</v>
-      </c>
-      <c r="G2" s="38" t="s">
-        <v>152</v>
+        <v>154</v>
+      </c>
+      <c r="D2" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="43" t="s">
+        <v>157</v>
+      </c>
+      <c r="G2" s="42" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E3" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F3" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="42" t="s">
         <v>155</v>
       </c>
-      <c r="G3" s="38" t="s">
-        <v>156</v>
+      <c r="E3" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F4" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="G4" s="38" t="s">
-        <v>160</v>
+        <v>163</v>
+      </c>
+      <c r="D4" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F4" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="G4" s="42" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F5" s="39" t="s">
-        <v>162</v>
-      </c>
-      <c r="G5" s="38" t="s">
-        <v>163</v>
+        <v>167</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F5" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F6" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="42" t="s">
         <v>164</v>
       </c>
-      <c r="G6" s="38" t="s">
-        <v>165</v>
+      <c r="F6" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="G6" s="42" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E7" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F7" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="G7" s="38" t="s">
         <v>167</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F7" s="43" t="s">
+        <v>172</v>
+      </c>
+      <c r="G7" s="42" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D8" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F8" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="G8" s="38" t="s">
-        <v>169</v>
+        <v>159</v>
+      </c>
+      <c r="D8" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E8" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8" s="42" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D9" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F9" s="39" t="s">
-        <v>171</v>
-      </c>
-      <c r="G9" s="38" t="s">
-        <v>172</v>
+        <v>176</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>177</v>
+      </c>
+      <c r="G9" s="42" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D10" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F10" s="39" t="s">
-        <v>174</v>
-      </c>
-      <c r="G10" s="38" t="s">
-        <v>175</v>
+        <v>179</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F10" s="43" t="s">
+        <v>180</v>
+      </c>
+      <c r="G10" s="42" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D11" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F11" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="G11" s="38" t="s">
-        <v>177</v>
+        <v>167</v>
+      </c>
+      <c r="D11" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F11" s="43" t="s">
+        <v>182</v>
+      </c>
+      <c r="G11" s="42" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D12" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E12" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F12" s="39" t="s">
-        <v>178</v>
-      </c>
-      <c r="G12" s="38" t="s">
-        <v>179</v>
+        <v>159</v>
+      </c>
+      <c r="D12" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E12" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F12" s="43" t="s">
+        <v>184</v>
+      </c>
+      <c r="G12" s="42" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D13" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F13" s="39" t="s">
-        <v>180</v>
-      </c>
-      <c r="G13" s="38" t="s">
-        <v>181</v>
+        <v>179</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E13" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F13" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="G13" s="42" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E14" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F14" s="39" t="s">
-        <v>182</v>
-      </c>
-      <c r="G14" s="38" t="s">
-        <v>183</v>
+        <v>176</v>
+      </c>
+      <c r="D14" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E14" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" s="42" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D15" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E15" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F15" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="G15" s="38" t="s">
-        <v>185</v>
+        <v>176</v>
+      </c>
+      <c r="D15" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="G15" s="42" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F16" s="39" t="s">
-        <v>186</v>
-      </c>
-      <c r="G16" s="38" t="s">
-        <v>187</v>
+        <v>179</v>
+      </c>
+      <c r="D16" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F16" s="43" t="s">
+        <v>192</v>
+      </c>
+      <c r="G16" s="42" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D17" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E17" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>189</v>
+        <v>176</v>
+      </c>
+      <c r="D17" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E17" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F17" s="43" t="s">
+        <v>194</v>
+      </c>
+      <c r="G17" s="42" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D18" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E18" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F18" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="G18" s="38" t="s">
-        <v>191</v>
+        <v>176</v>
+      </c>
+      <c r="D18" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E18" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>196</v>
+      </c>
+      <c r="G18" s="42" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D19" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>192</v>
-      </c>
-      <c r="G19" s="38" t="s">
-        <v>193</v>
+        <v>167</v>
+      </c>
+      <c r="D19" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="G19" s="42" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D20" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E20" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F20" s="39" t="s">
-        <v>194</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>195</v>
+        <v>159</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E20" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>200</v>
+      </c>
+      <c r="G20" s="42" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D21" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E21" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F21" s="39" t="s">
-        <v>196</v>
-      </c>
-      <c r="G21" s="38" t="s">
-        <v>197</v>
+        <v>176</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F21" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="G21" s="42" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D22" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E22" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F22" s="39" t="s">
-        <v>198</v>
-      </c>
-      <c r="G22" s="38" t="s">
-        <v>199</v>
+        <v>167</v>
+      </c>
+      <c r="D22" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E22" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>204</v>
+      </c>
+      <c r="G22" s="42" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>200</v>
-      </c>
-      <c r="G23" s="38" t="s">
-        <v>201</v>
+        <v>159</v>
+      </c>
+      <c r="D23" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E23" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>206</v>
+      </c>
+      <c r="G23" s="42" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D24" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E24" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F24" s="39" t="s">
-        <v>202</v>
-      </c>
-      <c r="G24" s="38" t="s">
-        <v>203</v>
+        <v>167</v>
+      </c>
+      <c r="D24" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E24" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F24" s="43" t="s">
+        <v>208</v>
+      </c>
+      <c r="G24" s="42" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E25" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F25" s="39" t="s">
-        <v>204</v>
-      </c>
-      <c r="G25" s="38" t="s">
-        <v>205</v>
+        <v>159</v>
+      </c>
+      <c r="D25" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F25" s="43" t="s">
+        <v>210</v>
+      </c>
+      <c r="G25" s="42" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D26" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E26" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F26" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="G26" s="38" t="s">
-        <v>207</v>
+        <v>167</v>
+      </c>
+      <c r="D26" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E26" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F26" s="43" t="s">
+        <v>212</v>
+      </c>
+      <c r="G26" s="42" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>208</v>
-      </c>
-      <c r="G27" s="38" t="s">
-        <v>209</v>
+        <v>159</v>
+      </c>
+      <c r="D27" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E27" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F27" s="43" t="s">
+        <v>214</v>
+      </c>
+      <c r="G27" s="42" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D28" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E28" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="39" t="s">
-        <v>210</v>
-      </c>
-      <c r="G28" s="38" t="s">
-        <v>211</v>
+        <v>179</v>
+      </c>
+      <c r="D28" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E28" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F28" s="43" t="s">
+        <v>216</v>
+      </c>
+      <c r="G28" s="42" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D29" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E29" s="38" t="s">
-        <v>158</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>212</v>
-      </c>
-      <c r="G29" s="38" t="s">
-        <v>213</v>
+        <v>176</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E29" s="42" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" s="43" t="s">
+        <v>218</v>
+      </c>
+      <c r="G29" s="42" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D30" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="E30" s="38" t="s">
-        <v>214</v>
-      </c>
-      <c r="F30" s="39" t="s">
-        <v>215</v>
-      </c>
-      <c r="G30" s="38" t="s">
-        <v>216</v>
+        <v>167</v>
+      </c>
+      <c r="D30" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E30" s="42" t="s">
+        <v>220</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="G30" s="42" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="B34" s="40" t="s">
-        <v>217</v>
+        <v>167</v>
+      </c>
+      <c r="B34" s="44" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>